<commit_message>
Agregar la talla final S-M-L-XL por etapa a Sizing_Behavioral_Design.xlsx
Nueva hoja "Resumen S-M-L-XL": un valor final por etapa y talla (no un
rango), con fila TOTAL (fórmula) y equivalencia en meses — mismo
formato que la tabla final acordada para el equipo. Vive junto a la
hoja granular (Hoja1) como su versión condensada de una sola pasada.
</commit_message>
<xml_diff>
--- a/reportes/Sizing_Behavioral_Design.xlsx
+++ b/reportes/Sizing_Behavioral_Design.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Resumen S-M-L-XL" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -123,7 +124,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -146,6 +147,18 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1252,4 +1265,216 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="27.125" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="10" t="inlineStr">
+        <is>
+          <t>ETAPA</t>
+        </is>
+      </c>
+      <c r="B1" s="11" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="C1" s="11" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="D1" s="11" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="E1" s="11" t="inlineStr">
+        <is>
+          <t>XL</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="12" t="inlineStr">
+        <is>
+          <t>Refinamiento</t>
+        </is>
+      </c>
+      <c r="B2" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="C2" s="13" t="n">
+        <v>6</v>
+      </c>
+      <c r="D2" s="13" t="n">
+        <v>8</v>
+      </c>
+      <c r="E2" s="13" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>Investigación</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="n">
+        <v>6</v>
+      </c>
+      <c r="C3" s="13" t="n">
+        <v>11</v>
+      </c>
+      <c r="D3" s="13" t="n">
+        <v>16</v>
+      </c>
+      <c r="E3" s="13" t="n">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
+          <t>Definición</t>
+        </is>
+      </c>
+      <c r="B4" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="C4" s="13" t="n">
+        <v>6</v>
+      </c>
+      <c r="D4" s="13" t="n">
+        <v>8</v>
+      </c>
+      <c r="E4" s="13" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>Diseño</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="n">
+        <v>6</v>
+      </c>
+      <c r="C5" s="13" t="n">
+        <v>9</v>
+      </c>
+      <c r="D5" s="13" t="n">
+        <v>14</v>
+      </c>
+      <c r="E5" s="13" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>Pruebas</t>
+        </is>
+      </c>
+      <c r="B6" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="C6" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="D6" s="13" t="n">
+        <v>6</v>
+      </c>
+      <c r="E6" s="13" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>Acompañamiento a la ejecución</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="n">
+        <v>5</v>
+      </c>
+      <c r="C7" s="13" t="n">
+        <v>6</v>
+      </c>
+      <c r="D7" s="13" t="n">
+        <v>8</v>
+      </c>
+      <c r="E7" s="13" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="10" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B8" s="11">
+        <f>SUM(B2:B7)</f>
+        <v/>
+      </c>
+      <c r="C8" s="11">
+        <f>SUM(C2:C7)</f>
+        <v/>
+      </c>
+      <c r="D8" s="11">
+        <f>SUM(D2:D7)</f>
+        <v/>
+      </c>
+      <c r="E8" s="11">
+        <f>SUM(E2:E7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>Equivalencia (meses)</t>
+        </is>
+      </c>
+      <c r="B9" s="11" t="inlineStr">
+        <is>
+          <t>1.4 m</t>
+        </is>
+      </c>
+      <c r="C9" s="11" t="inlineStr">
+        <is>
+          <t>2.1 m</t>
+        </is>
+      </c>
+      <c r="D9" s="11" t="inlineStr">
+        <is>
+          <t>3 m</t>
+        </is>
+      </c>
+      <c r="E9" s="11" t="inlineStr">
+        <is>
+          <t>6 m</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>